<commit_message>
add resultados de testes
</commit_message>
<xml_diff>
--- a/alocacao/saidas_2/resumo_custos.xlsx
+++ b/alocacao/saidas_2/resumo_custos.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -536,14 +536,14 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>01w24</t>
+          <t>00_350</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>48149</v>
+        <v>44309</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>230</v>
+        <v>315</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -551,42 +551,42 @@
         </is>
       </c>
       <c r="E3" s="3" t="n">
-        <v>2447547.16</v>
+        <v>2251792.29</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>2447547.16</v>
+        <v>2251796.97</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>2492096.56</v>
+        <v>2321788.93</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>1.82</v>
+        <v>3.11</v>
       </c>
       <c r="I3" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\01w24.csv</t>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\00_350.csv</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_2\alocacao_01w24</t>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_2\alocacao_00_350</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>10wLim</t>
+          <t>01w24</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>43864</v>
+        <v>48149</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>259</v>
+        <v>230</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -594,42 +594,42 @@
         </is>
       </c>
       <c r="E4" s="3" t="n">
-        <v>2228923.93</v>
+        <v>2447547.16</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>2228923.93</v>
+        <v>2447547.16</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>2261986.84</v>
+        <v>2492096.56</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>1.48</v>
+        <v>1.82</v>
       </c>
       <c r="I4" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\10wLim.csv</t>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\01w24.csv</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_2\alocacao_10wLim</t>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_2\alocacao_01w24</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>5072h</t>
+          <t>10wLim</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>46028</v>
+        <v>43864</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>202</v>
+        <v>259</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -637,42 +637,42 @@
         </is>
       </c>
       <c r="E5" s="3" t="n">
-        <v>2338453.5</v>
+        <v>2228923.93</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>2338459.2</v>
+        <v>2228923.93</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>2379435.43</v>
+        <v>2261986.84</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>1.75</v>
+        <v>1.48</v>
       </c>
       <c r="I5" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\5072h.csv</t>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\10wLim.csv</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_2\alocacao_5072h</t>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_2\alocacao_10wLim</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>50wLim</t>
+          <t>5072h</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>47400</v>
+        <v>46028</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>212</v>
+        <v>202</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -680,42 +680,42 @@
         </is>
       </c>
       <c r="E6" s="3" t="n">
-        <v>2409050.89</v>
+        <v>2338453.5</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>2409057.53</v>
+        <v>2338459.2</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>2450491.16</v>
+        <v>2379435.43</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>1.72</v>
+        <v>1.75</v>
       </c>
       <c r="I6" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\50wLim.csv</t>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\5072h.csv</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_2\alocacao_50wLim</t>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_2\alocacao_5072h</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>75w00</t>
+          <t>50wLim</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>49890</v>
+        <v>47400</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>227</v>
+        <v>212</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -723,42 +723,42 @@
         </is>
       </c>
       <c r="E7" s="3" t="n">
-        <v>2537623.54</v>
+        <v>2409050.89</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>2537623.54</v>
+        <v>2409057.53</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>2591364.94</v>
+        <v>2450491.16</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>2.12</v>
+        <v>1.72</v>
       </c>
       <c r="I7" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\75w00.csv</t>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\50wLim.csv</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_2\alocacao_75w00</t>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_2\alocacao_50wLim</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>heu_full</t>
+          <t>75w00</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>44127</v>
+        <v>49890</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>572</v>
+        <v>227</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -766,42 +766,42 @@
         </is>
       </c>
       <c r="E8" s="3" t="n">
-        <v>2244053.44</v>
+        <v>2537623.54</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>2244177.41</v>
+        <v>2537623.54</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>2583535.61</v>
+        <v>2591364.94</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>15.13</v>
+        <v>2.12</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\heu_full.csv</t>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\75w00.csv</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_2\alocacao_heu_full</t>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_2\alocacao_75w00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>heu_lim</t>
+          <t>heu_full</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>43812</v>
+        <v>44127</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>578</v>
+        <v>572</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -809,26 +809,69 @@
         </is>
       </c>
       <c r="E9" s="3" t="n">
-        <v>2226392.05</v>
+        <v>2244053.44</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>2226520.62</v>
+        <v>2244177.41</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>2549352.76</v>
+        <v>2583535.61</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>14.51</v>
+        <v>15.13</v>
       </c>
       <c r="I9" s="4" t="n">
         <v>0.01</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\heu_full.csv</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_2\alocacao_heu_full</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>heu_lim</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>43812</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>578</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>2226392.05</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>2226520.62</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>2549352.76</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>14.51</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\heu_lim.csv</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_2\alocacao_heu_lim</t>
         </is>

</xml_diff>

<commit_message>
Pequenas alteracoes e nos resultados e codigos do modeloIntegrado
</commit_message>
<xml_diff>
--- a/alocacao/saidas_2/resumo_custos.xlsx
+++ b/alocacao/saidas_2/resumo_custos.xlsx
@@ -55,13 +55,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -427,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M12"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -529,30 +531,20 @@
           <t>Sucesso</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2223257.66</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>2223489.44</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>2467920.5</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>11.0</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>0.01</t>
-        </is>
+      <c r="E2" s="4" t="n">
+        <v>2223257.66</v>
+      </c>
+      <c r="F2" s="4" t="n">
+        <v>2223489.44</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>2467920.5</v>
+      </c>
+      <c r="H2" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="I2" s="5" t="n">
+        <v>0.01</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -584,30 +576,20 @@
           <t>Sucesso</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2251792.29</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>2251796.97</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>2321788.93</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>3.11</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="E3" s="4" t="n">
+        <v>2251792.29</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>2251796.97</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>2321788.93</v>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>3.11</v>
+      </c>
+      <c r="I3" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -639,30 +621,20 @@
           <t>Sucesso</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2447547.16</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>2447547.16</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>2492096.56</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>1.82</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="E4" s="4" t="n">
+        <v>2447547.16</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>2447547.16</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>2492096.56</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="I4" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -694,30 +666,20 @@
           <t>Sucesso</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2228923.93</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>2228923.93</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2261986.84</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>1.48</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="E5" s="4" t="n">
+        <v>2228923.93</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>2228923.93</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>2261986.84</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="I5" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -749,30 +711,20 @@
           <t>Sucesso</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>2338453.5</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>2338459.2</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>2379435.43</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>1.75</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="E6" s="4" t="n">
+        <v>2338453.5</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>2338459.2</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>2379435.43</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="I6" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -804,30 +756,20 @@
           <t>Sucesso</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>2409050.89</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>2409057.53</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>2450491.16</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>1.72</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="E7" s="4" t="n">
+        <v>2409050.89</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>2409057.53</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>2450491.16</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="I7" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -859,30 +801,20 @@
           <t>Sucesso</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>2537623.54</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>2537623.54</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>2591364.94</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>2.12</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="E8" s="4" t="n">
+        <v>2537623.54</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>2537623.54</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>2591364.94</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="I8" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -914,30 +846,20 @@
           <t>Sucesso</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>2244053.44</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>2244177.41</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>2583535.61</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>15.13</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>0.01</t>
-        </is>
+      <c r="E9" s="4" t="n">
+        <v>2244053.44</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>2244177.41</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>2583535.61</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>15.13</v>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>0.01</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -969,30 +891,20 @@
           <t>Sucesso</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>2226392.05</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>2226520.62</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>2549352.76</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>14.51</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>0.01</t>
-        </is>
+      <c r="E10" s="4" t="n">
+        <v>2226392.05</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>2226520.62</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>2549352.76</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>14.51</v>
+      </c>
+      <c r="I10" s="5" t="n">
+        <v>0.01</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -1024,10 +936,8 @@
           <t>Sucesso (Sliding)</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>3021346.57</t>
-        </is>
+      <c r="E11" s="4" t="n">
+        <v>3021346.57</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
@@ -1038,10 +948,8 @@
       <c r="L11" t="n">
         <v>355</v>
       </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>3106454.93</t>
-        </is>
+      <c r="M11" s="4" t="n">
+        <v>3106454.93</v>
       </c>
     </row>
     <row r="12">
@@ -1061,10 +969,8 @@
           <t>Sucesso (Sliding)</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>2148117.95</t>
-        </is>
+      <c r="E12" s="4" t="n">
+        <v>2148117.95</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
@@ -1075,10 +981,107 @@
       <c r="L12" t="n">
         <v>318</v>
       </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>2465607.08</t>
-        </is>
+      <c r="M12" s="4" t="n">
+        <v>2465607.08</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>sliding_60_14_3</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>53510</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>538</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Sucesso (Sliding)</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>2722370.33</v>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="n">
+        <v>365</v>
+      </c>
+      <c r="M13" s="4" t="n">
+        <v>2722370.33</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>sliding_90_14_3</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>49560</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>592</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Sucesso (Sliding)</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>2526656.37</v>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="n">
+        <v>365</v>
+      </c>
+      <c r="M14" s="4" t="n">
+        <v>2526656.37</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>sliding_120_14_3</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>48518</v>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>581</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Sucesso (Sliding)</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>2466054.23</v>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="n">
+        <v>365</v>
+      </c>
+      <c r="M15" s="4" t="n">
+        <v>2466054.23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add coluna com os custos das entregas com a alocaoa original
</commit_message>
<xml_diff>
--- a/alocacao/saidas_2/resumo_custos.xlsx
+++ b/alocacao/saidas_2/resumo_custos.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M15"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -480,35 +480,40 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Custo Alocação Original</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Custo Heurística</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Gap Heurística vs M1 (%)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Gap M2 vs M1 (%)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Caminho da Entrada</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Pasta de Saída</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Qtd Dias</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Custo Projetado (365d)</t>
         </is>
@@ -538,26 +543,27 @@
         <v>2223489.44</v>
       </c>
       <c r="G2" s="4" t="n">
+        <v>2845265.79</v>
+      </c>
+      <c r="H2" s="4" t="n">
         <v>2467920.5</v>
       </c>
-      <c r="H2" s="5" t="n">
+      <c r="I2" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="I2" s="5" t="n">
+      <c r="J2" s="5" t="n">
         <v>0.01</v>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\00.csv</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_2\alocacao_00</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -583,26 +589,27 @@
         <v>2251796.97</v>
       </c>
       <c r="G3" s="4" t="n">
+        <v>2880644.2</v>
+      </c>
+      <c r="H3" s="4" t="n">
         <v>2321788.93</v>
       </c>
-      <c r="H3" s="5" t="n">
+      <c r="I3" s="5" t="n">
         <v>3.11</v>
       </c>
-      <c r="I3" s="5" t="n">
+      <c r="J3" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\00_350.csv</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_2\alocacao_00_350</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -628,26 +635,27 @@
         <v>2447547.16</v>
       </c>
       <c r="G4" s="4" t="n">
+        <v>3128675.16</v>
+      </c>
+      <c r="H4" s="4" t="n">
         <v>2492096.56</v>
       </c>
-      <c r="H4" s="5" t="n">
+      <c r="I4" s="5" t="n">
         <v>1.82</v>
       </c>
-      <c r="I4" s="5" t="n">
+      <c r="J4" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\01w24.csv</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_2\alocacao_01w24</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -673,26 +681,27 @@
         <v>2228923.93</v>
       </c>
       <c r="G5" s="4" t="n">
+        <v>2853328.28</v>
+      </c>
+      <c r="H5" s="4" t="n">
         <v>2261986.84</v>
       </c>
-      <c r="H5" s="5" t="n">
+      <c r="I5" s="5" t="n">
         <v>1.48</v>
       </c>
-      <c r="I5" s="5" t="n">
+      <c r="J5" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\10wLim.csv</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_2\alocacao_10wLim</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -718,26 +727,27 @@
         <v>2338459.2</v>
       </c>
       <c r="G6" s="4" t="n">
+        <v>2992393.1</v>
+      </c>
+      <c r="H6" s="4" t="n">
         <v>2379435.43</v>
       </c>
-      <c r="H6" s="5" t="n">
+      <c r="I6" s="5" t="n">
         <v>1.75</v>
       </c>
-      <c r="I6" s="5" t="n">
+      <c r="J6" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\5072h.csv</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_2\alocacao_5072h</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -763,26 +773,27 @@
         <v>2409057.53</v>
       </c>
       <c r="G7" s="4" t="n">
+        <v>3082488.75</v>
+      </c>
+      <c r="H7" s="4" t="n">
         <v>2450491.16</v>
       </c>
-      <c r="H7" s="5" t="n">
+      <c r="I7" s="5" t="n">
         <v>1.72</v>
       </c>
-      <c r="I7" s="5" t="n">
+      <c r="J7" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\50wLim.csv</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_2\alocacao_50wLim</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -808,26 +819,27 @@
         <v>2537623.54</v>
       </c>
       <c r="G8" s="4" t="n">
+        <v>3241183.97</v>
+      </c>
+      <c r="H8" s="4" t="n">
         <v>2591364.94</v>
       </c>
-      <c r="H8" s="5" t="n">
+      <c r="I8" s="5" t="n">
         <v>2.12</v>
       </c>
-      <c r="I8" s="5" t="n">
+      <c r="J8" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\75w00.csv</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_2\alocacao_75w00</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -853,26 +865,27 @@
         <v>2244177.41</v>
       </c>
       <c r="G9" s="4" t="n">
+        <v>2879155.22</v>
+      </c>
+      <c r="H9" s="4" t="n">
         <v>2583535.61</v>
       </c>
-      <c r="H9" s="5" t="n">
+      <c r="I9" s="5" t="n">
         <v>15.13</v>
       </c>
-      <c r="I9" s="5" t="n">
+      <c r="J9" s="5" t="n">
         <v>0.01</v>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\heu_full.csv</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_2\alocacao_heu_full</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -898,26 +911,27 @@
         <v>2226520.62</v>
       </c>
       <c r="G10" s="4" t="n">
+        <v>2849433.23</v>
+      </c>
+      <c r="H10" s="4" t="n">
         <v>2549352.76</v>
       </c>
-      <c r="H10" s="5" t="n">
+      <c r="I10" s="5" t="n">
         <v>14.51</v>
       </c>
-      <c r="I10" s="5" t="n">
+      <c r="J10" s="5" t="n">
         <v>0.01</v>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\heu_lim.csv</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_2\alocacao_heu_lim</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -939,16 +953,10 @@
       <c r="E11" s="4" t="n">
         <v>3021346.57</v>
       </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="n">
+      <c r="M11" t="n">
         <v>355</v>
       </c>
-      <c r="M11" s="4" t="n">
+      <c r="N11" s="4" t="n">
         <v>3106454.93</v>
       </c>
     </row>
@@ -972,16 +980,10 @@
       <c r="E12" s="4" t="n">
         <v>2148117.95</v>
       </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="n">
+      <c r="M12" t="n">
         <v>318</v>
       </c>
-      <c r="M12" s="4" t="n">
+      <c r="N12" s="4" t="n">
         <v>2465607.08</v>
       </c>
     </row>
@@ -1005,16 +1007,10 @@
       <c r="E13" s="4" t="n">
         <v>2722370.33</v>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="n">
+      <c r="M13" t="n">
         <v>365</v>
       </c>
-      <c r="M13" s="4" t="n">
+      <c r="N13" s="4" t="n">
         <v>2722370.33</v>
       </c>
     </row>
@@ -1038,16 +1034,10 @@
       <c r="E14" s="4" t="n">
         <v>2526656.37</v>
       </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="n">
+      <c r="M14" t="n">
         <v>365</v>
       </c>
-      <c r="M14" s="4" t="n">
+      <c r="N14" s="4" t="n">
         <v>2526656.37</v>
       </c>
     </row>
@@ -1071,16 +1061,10 @@
       <c r="E15" s="4" t="n">
         <v>2466054.23</v>
       </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="n">
+      <c r="M15" t="n">
         <v>365</v>
       </c>
-      <c r="M15" s="4" t="n">
+      <c r="N15" s="4" t="n">
         <v>2466054.23</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: fix on m1 for repeat tests
</commit_message>
<xml_diff>
--- a/alocacao/saidas_2/resumo_custos.xlsx
+++ b/alocacao/saidas_2/resumo_custos.xlsx
@@ -429,22 +429,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:W15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="34" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="27" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
-    <col width="92" customWidth="1" min="10" max="10"/>
-    <col width="97" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="25" customWidth="1" min="13" max="13"/>
+    <col width="32" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
+    <col width="34" customWidth="1" min="13" max="13"/>
+    <col width="33" customWidth="1" min="14" max="14"/>
+    <col width="27" customWidth="1" min="15" max="15"/>
+    <col width="32" customWidth="1" min="16" max="16"/>
+    <col width="31" customWidth="1" min="17" max="17"/>
+    <col width="25" customWidth="1" min="18" max="18"/>
+    <col width="33" customWidth="1" min="19" max="19"/>
+    <col width="92" customWidth="1" min="20" max="20"/>
+    <col width="97" customWidth="1" min="21" max="21"/>
+    <col width="11" customWidth="1" min="22" max="22"/>
+    <col width="25" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -470,50 +480,95 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Custo Modelo Exato (M1)</t>
+          <t>Custo M1 Diário</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Custo M1 Anual</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Custo Modelo Anual (M2)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Custo Alocação Original</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Custo Heurística</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Gap Heurística vs M1 (%)</t>
-        </is>
-      </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Gap M2 vs M1 (%)</t>
+          <t>Gap M1 Anual vs M1 Diário (%)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>Gap M2 vs M1 Diário (%)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Gap M2 vs M1 Anual (%)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Gap Heurística vs M1 Diário (%)</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Gap Heurística vs M1 Anual (%)</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Gap Heurística vs M2 (%)</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Gap Original vs M1 Diário (%)</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Gap Original vs M1 Anual (%)</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Gap Original vs M2 (%)</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Gap Original vs Heurística (%)</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
           <t>Caminho da Entrada</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Pasta de Saída</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Qtd Dias</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Custo Projetado (365d)</t>
         </is>
@@ -540,30 +595,59 @@
         <v>2223257.66</v>
       </c>
       <c r="F2" s="4" t="n">
+        <v>1651961.02</v>
+      </c>
+      <c r="G2" s="4" t="n">
         <v>2223489.44</v>
       </c>
-      <c r="G2" s="4" t="n">
+      <c r="H2" s="4" t="n">
         <v>2845265.79</v>
       </c>
-      <c r="H2" s="4" t="n">
+      <c r="I2" s="4" t="n">
         <v>2467920.5</v>
       </c>
-      <c r="I2" s="5" t="n">
+      <c r="J2" s="5" t="n">
+        <v>-25.7</v>
+      </c>
+      <c r="K2" s="5" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="L2" s="5" t="n">
+        <v>34.6</v>
+      </c>
+      <c r="M2" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="J2" s="5" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="K2" t="inlineStr">
+      <c r="N2" s="5" t="n">
+        <v>49.39</v>
+      </c>
+      <c r="O2" s="5" t="n">
+        <v>10.99</v>
+      </c>
+      <c r="P2" s="5" t="n">
+        <v>27.98</v>
+      </c>
+      <c r="Q2" s="5" t="n">
+        <v>72.23999999999999</v>
+      </c>
+      <c r="R2" s="5" t="n">
+        <v>27.96</v>
+      </c>
+      <c r="S2" s="5" t="n">
+        <v>15.29</v>
+      </c>
+      <c r="T2" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\00.csv</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_2\alocacao_00</t>
         </is>
       </c>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -586,30 +670,59 @@
         <v>2251792.29</v>
       </c>
       <c r="F3" s="4" t="n">
+        <v>1631784.92</v>
+      </c>
+      <c r="G3" s="4" t="n">
         <v>2251796.97</v>
       </c>
-      <c r="G3" s="4" t="n">
+      <c r="H3" s="4" t="n">
         <v>2880644.2</v>
       </c>
-      <c r="H3" s="4" t="n">
+      <c r="I3" s="4" t="n">
         <v>2321788.93</v>
       </c>
-      <c r="I3" s="5" t="n">
+      <c r="J3" s="5" t="n">
+        <v>-27.53</v>
+      </c>
+      <c r="K3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="M3" s="5" t="n">
         <v>3.11</v>
       </c>
-      <c r="J3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="inlineStr">
+      <c r="N3" s="5" t="n">
+        <v>42.29</v>
+      </c>
+      <c r="O3" s="5" t="n">
+        <v>3.11</v>
+      </c>
+      <c r="P3" s="5" t="n">
+        <v>27.93</v>
+      </c>
+      <c r="Q3" s="5" t="n">
+        <v>76.53</v>
+      </c>
+      <c r="R3" s="5" t="n">
+        <v>27.93</v>
+      </c>
+      <c r="S3" s="5" t="n">
+        <v>24.07</v>
+      </c>
+      <c r="T3" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\00_350.csv</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_2\alocacao_00_350</t>
         </is>
       </c>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -632,30 +745,59 @@
         <v>2447547.16</v>
       </c>
       <c r="F4" s="4" t="n">
+        <v>1769937.39</v>
+      </c>
+      <c r="G4" s="4" t="n">
         <v>2447547.16</v>
       </c>
-      <c r="G4" s="4" t="n">
+      <c r="H4" s="4" t="n">
         <v>3128675.16</v>
       </c>
-      <c r="H4" s="4" t="n">
+      <c r="I4" s="4" t="n">
         <v>2492096.56</v>
       </c>
-      <c r="I4" s="5" t="n">
+      <c r="J4" s="5" t="n">
+        <v>-27.69</v>
+      </c>
+      <c r="K4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="5" t="n">
+        <v>38.28</v>
+      </c>
+      <c r="M4" s="5" t="n">
         <v>1.82</v>
       </c>
-      <c r="J4" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="inlineStr">
+      <c r="N4" s="5" t="n">
+        <v>40.8</v>
+      </c>
+      <c r="O4" s="5" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="P4" s="5" t="n">
+        <v>27.83</v>
+      </c>
+      <c r="Q4" s="5" t="n">
+        <v>76.77</v>
+      </c>
+      <c r="R4" s="5" t="n">
+        <v>27.83</v>
+      </c>
+      <c r="S4" s="5" t="n">
+        <v>25.54</v>
+      </c>
+      <c r="T4" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\01w24.csv</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_2\alocacao_01w24</t>
         </is>
       </c>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -678,30 +820,59 @@
         <v>2228923.93</v>
       </c>
       <c r="F5" s="4" t="n">
+        <v>1608397.4</v>
+      </c>
+      <c r="G5" s="4" t="n">
         <v>2228923.93</v>
       </c>
-      <c r="G5" s="4" t="n">
+      <c r="H5" s="4" t="n">
         <v>2853328.28</v>
       </c>
-      <c r="H5" s="4" t="n">
+      <c r="I5" s="4" t="n">
         <v>2261986.84</v>
       </c>
-      <c r="I5" s="5" t="n">
+      <c r="J5" s="5" t="n">
+        <v>-27.84</v>
+      </c>
+      <c r="K5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="5" t="n">
+        <v>38.58</v>
+      </c>
+      <c r="M5" s="5" t="n">
         <v>1.48</v>
       </c>
-      <c r="J5" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="inlineStr">
+      <c r="N5" s="5" t="n">
+        <v>40.64</v>
+      </c>
+      <c r="O5" s="5" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="P5" s="5" t="n">
+        <v>28.01</v>
+      </c>
+      <c r="Q5" s="5" t="n">
+        <v>77.40000000000001</v>
+      </c>
+      <c r="R5" s="5" t="n">
+        <v>28.01</v>
+      </c>
+      <c r="S5" s="5" t="n">
+        <v>26.14</v>
+      </c>
+      <c r="T5" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\10wLim.csv</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_2\alocacao_10wLim</t>
         </is>
       </c>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -724,30 +895,59 @@
         <v>2338453.5</v>
       </c>
       <c r="F6" s="4" t="n">
+        <v>1691970.72</v>
+      </c>
+      <c r="G6" s="4" t="n">
         <v>2338459.2</v>
       </c>
-      <c r="G6" s="4" t="n">
+      <c r="H6" s="4" t="n">
         <v>2992393.1</v>
       </c>
-      <c r="H6" s="4" t="n">
+      <c r="I6" s="4" t="n">
         <v>2379435.43</v>
       </c>
-      <c r="I6" s="5" t="n">
+      <c r="J6" s="5" t="n">
+        <v>-27.65</v>
+      </c>
+      <c r="K6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="5" t="n">
+        <v>38.21</v>
+      </c>
+      <c r="M6" s="5" t="n">
         <v>1.75</v>
       </c>
-      <c r="J6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="inlineStr">
+      <c r="N6" s="5" t="n">
+        <v>40.63</v>
+      </c>
+      <c r="O6" s="5" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="P6" s="5" t="n">
+        <v>27.96</v>
+      </c>
+      <c r="Q6" s="5" t="n">
+        <v>76.86</v>
+      </c>
+      <c r="R6" s="5" t="n">
+        <v>27.96</v>
+      </c>
+      <c r="S6" s="5" t="n">
+        <v>25.76</v>
+      </c>
+      <c r="T6" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\5072h.csv</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_2\alocacao_5072h</t>
         </is>
       </c>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -770,30 +970,59 @@
         <v>2409050.89</v>
       </c>
       <c r="F7" s="4" t="n">
+        <v>1742818.55</v>
+      </c>
+      <c r="G7" s="4" t="n">
         <v>2409057.53</v>
       </c>
-      <c r="G7" s="4" t="n">
+      <c r="H7" s="4" t="n">
         <v>3082488.75</v>
       </c>
-      <c r="H7" s="4" t="n">
+      <c r="I7" s="4" t="n">
         <v>2450491.16</v>
       </c>
-      <c r="I7" s="5" t="n">
+      <c r="J7" s="5" t="n">
+        <v>-27.66</v>
+      </c>
+      <c r="K7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="5" t="n">
+        <v>38.23</v>
+      </c>
+      <c r="M7" s="5" t="n">
         <v>1.72</v>
       </c>
-      <c r="J7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" t="inlineStr">
+      <c r="N7" s="5" t="n">
+        <v>40.61</v>
+      </c>
+      <c r="O7" s="5" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="P7" s="5" t="n">
+        <v>27.95</v>
+      </c>
+      <c r="Q7" s="5" t="n">
+        <v>76.87</v>
+      </c>
+      <c r="R7" s="5" t="n">
+        <v>27.95</v>
+      </c>
+      <c r="S7" s="5" t="n">
+        <v>25.79</v>
+      </c>
+      <c r="T7" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\50wLim.csv</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_2\alocacao_50wLim</t>
         </is>
       </c>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -816,30 +1045,59 @@
         <v>2537623.54</v>
       </c>
       <c r="F8" s="4" t="n">
+        <v>1833876.28</v>
+      </c>
+      <c r="G8" s="4" t="n">
         <v>2537623.54</v>
       </c>
-      <c r="G8" s="4" t="n">
+      <c r="H8" s="4" t="n">
         <v>3241183.97</v>
       </c>
-      <c r="H8" s="4" t="n">
+      <c r="I8" s="4" t="n">
         <v>2591364.94</v>
       </c>
-      <c r="I8" s="5" t="n">
+      <c r="J8" s="5" t="n">
+        <v>-27.73</v>
+      </c>
+      <c r="K8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="5" t="n">
+        <v>38.37</v>
+      </c>
+      <c r="M8" s="5" t="n">
         <v>2.12</v>
       </c>
-      <c r="J8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" t="inlineStr">
+      <c r="N8" s="5" t="n">
+        <v>41.31</v>
+      </c>
+      <c r="O8" s="5" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="P8" s="5" t="n">
+        <v>27.73</v>
+      </c>
+      <c r="Q8" s="5" t="n">
+        <v>76.73999999999999</v>
+      </c>
+      <c r="R8" s="5" t="n">
+        <v>27.73</v>
+      </c>
+      <c r="S8" s="5" t="n">
+        <v>25.08</v>
+      </c>
+      <c r="T8" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\75w00.csv</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="U8" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_2\alocacao_75w00</t>
         </is>
       </c>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -862,30 +1120,59 @@
         <v>2244053.44</v>
       </c>
       <c r="F9" s="4" t="n">
+        <v>1678633.51</v>
+      </c>
+      <c r="G9" s="4" t="n">
         <v>2244177.41</v>
       </c>
-      <c r="G9" s="4" t="n">
+      <c r="H9" s="4" t="n">
         <v>2879155.22</v>
       </c>
-      <c r="H9" s="4" t="n">
+      <c r="I9" s="4" t="n">
         <v>2583535.61</v>
       </c>
-      <c r="I9" s="5" t="n">
+      <c r="J9" s="5" t="n">
+        <v>-25.2</v>
+      </c>
+      <c r="K9" s="5" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="L9" s="5" t="n">
+        <v>33.69</v>
+      </c>
+      <c r="M9" s="5" t="n">
         <v>15.13</v>
       </c>
-      <c r="J9" s="5" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="K9" t="inlineStr">
+      <c r="N9" s="5" t="n">
+        <v>53.91</v>
+      </c>
+      <c r="O9" s="5" t="n">
+        <v>15.12</v>
+      </c>
+      <c r="P9" s="5" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="Q9" s="5" t="n">
+        <v>71.52</v>
+      </c>
+      <c r="R9" s="5" t="n">
+        <v>28.29</v>
+      </c>
+      <c r="S9" s="5" t="n">
+        <v>11.44</v>
+      </c>
+      <c r="T9" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\heu_full.csv</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="U9" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_2\alocacao_heu_full</t>
         </is>
       </c>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -908,30 +1195,59 @@
         <v>2226392.05</v>
       </c>
       <c r="F10" s="4" t="n">
+        <v>1653185.87</v>
+      </c>
+      <c r="G10" s="4" t="n">
         <v>2226520.62</v>
       </c>
-      <c r="G10" s="4" t="n">
+      <c r="H10" s="4" t="n">
         <v>2849433.23</v>
       </c>
-      <c r="H10" s="4" t="n">
+      <c r="I10" s="4" t="n">
         <v>2549352.76</v>
       </c>
-      <c r="I10" s="5" t="n">
+      <c r="J10" s="5" t="n">
+        <v>-25.75</v>
+      </c>
+      <c r="K10" s="5" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="L10" s="5" t="n">
+        <v>34.68</v>
+      </c>
+      <c r="M10" s="5" t="n">
         <v>14.51</v>
       </c>
-      <c r="J10" s="5" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="K10" t="inlineStr">
+      <c r="N10" s="5" t="n">
+        <v>54.21</v>
+      </c>
+      <c r="O10" s="5" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="P10" s="5" t="n">
+        <v>27.98</v>
+      </c>
+      <c r="Q10" s="5" t="n">
+        <v>72.36</v>
+      </c>
+      <c r="R10" s="5" t="n">
+        <v>27.98</v>
+      </c>
+      <c r="S10" s="5" t="n">
+        <v>11.77</v>
+      </c>
+      <c r="T10" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\heu_lim.csv</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="U10" t="inlineStr">
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_2\alocacao_heu_lim</t>
         </is>
       </c>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -953,10 +1269,26 @@
       <c r="E11" s="4" t="n">
         <v>3021346.57</v>
       </c>
-      <c r="M11" t="n">
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="n">
         <v>355</v>
       </c>
-      <c r="N11" s="4" t="n">
+      <c r="W11" s="4" t="n">
         <v>3106454.93</v>
       </c>
     </row>
@@ -980,10 +1312,26 @@
       <c r="E12" s="4" t="n">
         <v>2148117.95</v>
       </c>
-      <c r="M12" t="n">
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="n">
         <v>318</v>
       </c>
-      <c r="N12" s="4" t="n">
+      <c r="W12" s="4" t="n">
         <v>2465607.08</v>
       </c>
     </row>
@@ -1007,10 +1355,26 @@
       <c r="E13" s="4" t="n">
         <v>2722370.33</v>
       </c>
-      <c r="M13" t="n">
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr"/>
+      <c r="V13" t="n">
         <v>365</v>
       </c>
-      <c r="N13" s="4" t="n">
+      <c r="W13" s="4" t="n">
         <v>2722370.33</v>
       </c>
     </row>
@@ -1034,10 +1398,26 @@
       <c r="E14" s="4" t="n">
         <v>2526656.37</v>
       </c>
-      <c r="M14" t="n">
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="n">
         <v>365</v>
       </c>
-      <c r="N14" s="4" t="n">
+      <c r="W14" s="4" t="n">
         <v>2526656.37</v>
       </c>
     </row>
@@ -1061,10 +1441,26 @@
       <c r="E15" s="4" t="n">
         <v>2466054.23</v>
       </c>
-      <c r="M15" t="n">
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="n">
         <v>365</v>
       </c>
-      <c r="N15" s="4" t="n">
+      <c r="W15" s="4" t="n">
         <v>2466054.23</v>
       </c>
     </row>

</xml_diff>